<commit_message>
A felicidade está online :)
</commit_message>
<xml_diff>
--- a/PythonCodes/Results/validacao_modelos.xlsx
+++ b/PythonCodes/Results/validacao_modelos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Por_atleta" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Por_atleta" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,47 +418,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Grupo</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Tempo_real_h</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Pot_prev_h</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Sig_prev_h</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Hyper_prev_h</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Erro%_Pot</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Erro%_Sig</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Erro%_Hyper</t>
         </is>
@@ -593,7 +581,7 @@
         <v>-3.078268951093646</v>
       </c>
       <c r="H4" t="n">
-        <v>13.99231806127598</v>
+        <v>13.98957073088863</v>
       </c>
       <c r="I4" t="n">
         <v>15.46796548294589</v>
@@ -745,7 +733,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4:37:04</t>
+          <t>4:37:14</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -753,7 +741,7 @@
         <v>-5.88449224383744</v>
       </c>
       <c r="H8" t="n">
-        <v>41.73304773432</v>
+        <v>41.82149454276675</v>
       </c>
       <c r="I8" t="inlineStr"/>
     </row>
@@ -836,7 +824,7 @@
         <v>-3.718735771926269</v>
       </c>
       <c r="I10" t="n">
-        <v>8.071446502139917</v>
+        <v>8.071403354171851</v>
       </c>
     </row>
     <row r="11">
@@ -1205,7 +1193,7 @@
         <v>-8.042370278065601</v>
       </c>
       <c r="I19" t="n">
-        <v>1.951113047562244</v>
+        <v>1.951144135843109</v>
       </c>
     </row>
     <row r="20">
@@ -1246,7 +1234,7 @@
         <v>-6.536555689722162</v>
       </c>
       <c r="I20" t="n">
-        <v>5.941191226140325</v>
+        <v>5.941160019914669</v>
       </c>
     </row>
     <row r="21">
@@ -1674,19 +1662,19 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>MAPE_% (erro absoluto médio)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Vies_% (erro médio com sinal)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Potencia</t>
         </is>
@@ -1699,20 +1687,20 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Sigmoide</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9.076000000000001</v>
+        <v>9.079000000000001</v>
       </c>
       <c r="C3" t="n">
-        <v>-4.384</v>
+        <v>-4.381</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Hyper</t>
         </is>

</xml_diff>